<commit_message>
Course Assignment & Industry Consultant: Emeritus stays available, faculty dropdowns mirror the Faculty list
- Re-validate icon button restored on the Course Assignment page
- Emeritus course assignments stay visible/flagged (red pill) instead of being archived; only Inactive/Archived route to the Archive
- Upload warning + controller docs updated to reflect Emeritus = available for reassignment
- Faculty dropdowns on Course Assignment and Industry Consultant now exclude archived (Emeritus/Inactive) faculty, mirroring the Faculty list
</commit_message>
<xml_diff>
--- a/sample-uploads/sample_course_assignments.xlsx
+++ b/sample-uploads/sample_course_assignments.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,16 +418,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BIT201</v>
+        <v>BIT101</v>
       </c>
       <c r="B2" t="str">
-        <v>Database Systems</v>
+        <v>Introduction to Computing</v>
       </c>
       <c r="C2" t="str">
-        <v>2nd Year</v>
+        <v>1st Year</v>
       </c>
       <c r="D2" t="str">
-        <v>Marceline Avila</v>
+        <v>Bianca G. Reyes</v>
       </c>
       <c r="E2" t="str">
         <v>2027-08-18</v>
@@ -435,16 +435,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BIT202</v>
+        <v>BIT102</v>
       </c>
       <c r="B3" t="str">
-        <v>Software Engineering</v>
+        <v>Computer Programming 1</v>
       </c>
       <c r="C3" t="str">
-        <v>3rd Year</v>
+        <v>1st Year</v>
       </c>
       <c r="D3" t="str">
-        <v>Dennis Ignacio</v>
+        <v>Bowen Higgins</v>
       </c>
       <c r="E3" t="str">
         <v>2027-08-18</v>
@@ -452,16 +452,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BIT203</v>
+        <v>BIT201</v>
       </c>
       <c r="B4" t="str">
-        <v>Mobile Application Development</v>
+        <v>Database Systems</v>
       </c>
       <c r="C4" t="str">
-        <v>3rd Year</v>
+        <v>2nd Year</v>
       </c>
       <c r="D4" t="str">
-        <v>Bianca G. Reyes</v>
+        <v>Marceline Avila</v>
       </c>
       <c r="E4" t="str">
         <v>2027-08-18</v>
@@ -469,16 +469,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BIT204</v>
+        <v>BIT202</v>
       </c>
       <c r="B5" t="str">
-        <v>Network Security</v>
+        <v>Object-Oriented Programming</v>
       </c>
       <c r="C5" t="str">
-        <v>3rd Year</v>
+        <v>2nd Year</v>
       </c>
       <c r="D5" t="str">
-        <v>Danny B. Casimero</v>
+        <v>Christine A. Dizon</v>
       </c>
       <c r="E5" t="str">
         <v>2027-08-18</v>
@@ -495,7 +495,7 @@
         <v>2nd Year</v>
       </c>
       <c r="D6" t="str">
-        <v>Bowen Higgins</v>
+        <v>Dennis Ignacio</v>
       </c>
       <c r="E6" t="str">
         <v>2027-08-18</v>
@@ -503,10 +503,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BIT206</v>
+        <v>BIT301</v>
       </c>
       <c r="B7" t="str">
-        <v>Introduction to Artificial Intelligence</v>
+        <v>Web Development</v>
       </c>
       <c r="C7" t="str">
         <v>3rd Year</v>
@@ -520,16 +520,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BIT207</v>
+        <v>BIT303</v>
       </c>
       <c r="B8" t="str">
-        <v>Web Security and Performance</v>
+        <v>Software Engineering</v>
       </c>
       <c r="C8" t="str">
         <v>3rd Year</v>
       </c>
       <c r="D8" t="str">
-        <v>Michael R. Lee</v>
+        <v>Danny B. Casimero</v>
       </c>
       <c r="E8" t="str">
         <v>2027-08-18</v>
@@ -537,16 +537,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BIT302</v>
+        <v>BIT304</v>
       </c>
       <c r="B9" t="str">
-        <v>Web Development II</v>
+        <v>Network Security</v>
       </c>
       <c r="C9" t="str">
-        <v>2nd Year</v>
+        <v>3rd Year</v>
       </c>
       <c r="D9" t="str">
-        <v>Christine A. Dizon</v>
+        <v>Michael R. Lee</v>
       </c>
       <c r="E9" t="str">
         <v>2027-08-18</v>
@@ -569,9 +569,26 @@
         <v>2027-08-18</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>BIT401</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Capstone Project 1</v>
+      </c>
+      <c r="C11" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Danny B. Casimero</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2027-08-18</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>